<commit_message>
Dark header band, drop live clock, rename In Transit -> Sailing
- Header is now a full-bleed dark navy band (logo sits on a white
  plate since the source PNG has no transparency), title in white,
  REF TIME/TRACKING chip restyled for the dark background.
- Remove the live real-time clock (added in a prior session) per
  request -- it's redundant with REF TIME (from file).
- "In transit" status is now labelled "Sailing" throughout (status
  pill, filter chip, legend); internal 'transit' identifiers unchanged.

Regenerated Vessel Schedule.html/.xlsx from the existing sked_current/
sked_prev state (not a new --full run) so the Early/Delay baseline
against 9-11-1600 is preserved.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Vessel Schedule.xlsx
+++ b/Vessel Schedule.xlsx
@@ -1069,20 +1069,22 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>nodata</t>
+          <t>docked</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="n">
-        <v/>
+          <t>KRPUS (PUSH4)</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>2607S</t>
+        </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>No data in window</t>
+          <t>Alongside, departs to KRUSN ~2026-09-14T20:30:00</t>
         </is>
       </c>
       <c r="I10" s="3" t="n"/>

</xml_diff>

<commit_message>
Remove mobile preview; add a Calendar view
- Drop the Desktop/Mobile toggle and iframe-based phone preview
  entirely (CSS, HTML, and JS).
- Add a List/Calendar view switch, moved down into the page flow
  (below search/filters, above the results) instead of sitting above
  the header like the old toggle did.
- Calendar is a month grid built from every THBKK/THLCH leg across
  all vessels (not just each vessel's next call), with prev/next/
  Today navigation, a per-day chip list (color-coded by port), and a
  click-to-expand detail panel listing full time/wharf per call.
  Respects the existing vessel-name search.

Regenerated from the existing sked_current/sked_prev state (not a
new --full run) so the Early/Delay baseline is preserved.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Vessel Schedule.xlsx
+++ b/Vessel Schedule.xlsx
@@ -1135,22 +1135,20 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>docked</t>
+          <t>transit</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>VNSGN (SGN03)</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="inlineStr">
-        <is>
-          <t>2611S</t>
-        </is>
+          <t>VNSGN -&gt; THLCH</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="n">
+        <v/>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>Alongside, departs to THLCH ~2026-09-16T16:00:00</t>
+          <t>In transit, ETA 2026-09-18T10:00:00</t>
         </is>
       </c>
       <c r="I11" s="3" t="n">
@@ -1515,20 +1513,22 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>nodata</t>
+          <t>docked</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G17" s="2" t="n">
-        <v/>
+          <t>KRPUS (PUS05)</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>2608S</t>
+        </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>No data in window</t>
+          <t>Alongside, departs to KRINC ~2026-09-17T21:00:00</t>
         </is>
       </c>
       <c r="I17" s="3" t="n">

</xml_diff>

<commit_message>
Calendar detail: show vessel short code before the full name
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Vessel Schedule.xlsx
+++ b/Vessel Schedule.xlsx
@@ -2101,20 +2101,22 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>nodata</t>
+          <t>docked</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G26" s="2" t="n">
-        <v/>
+          <t>THLCH (LCH04)</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>2610S</t>
+        </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>No data in window</t>
+          <t>Alongside, departs to THBKK ~2026-09-17T00:00:00</t>
         </is>
       </c>
       <c r="I26" s="3" t="n">
@@ -2131,7 +2133,7 @@
         </is>
       </c>
       <c r="L26" s="3" t="n">
-        <v>46281.70833333334</v>
+        <v>46283.95833333334</v>
       </c>
       <c r="M26" s="2" t="inlineStr">
         <is>
@@ -2140,7 +2142,7 @@
       </c>
       <c r="N26" s="2" t="inlineStr">
         <is>
-          <t>2610S</t>
+          <t>2610N</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix dashboard clock using UTC instead of Bangkok time on auto-runs
GitHub Actions runners use UTC system time, but generate_vessel_schedule.py
called datetime.now() without a timezone whenever --now wasn't passed. The
dashboard then rendered that UTC value as if it were Bangkok local time
(since ETA/ETB/ETD are naive Bangkok-local and rendered the same way),
making the header clock -- and the alongside/sailing/countdown logic that
depends on "now" -- run 7 hours behind whenever an auto-fetch generated
the page. Manual runs from a Bangkok-timezone PC were unaffected.

Also regenerates the currently published dashboard with the corrected
time so the live site isn't stuck showing a UTC-mislabeled clock until
the next scheduled run.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Vessel Schedule.xlsx
+++ b/Vessel Schedule.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Full Schedule" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Early-Delay" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Full Schedule" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Early-Delay" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1043,22 +1043,20 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>docked</t>
+          <t>transit</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>THBKK (BKK01)</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="inlineStr">
-        <is>
-          <t>2610N</t>
-        </is>
+          <t>THBKK -&gt; THLCH</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="n">
+        <v/>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Alongside, departs to THLCH ~2026-09-24T12:00:00</t>
+          <t>In transit, ETA 2026-09-24T17:00:00</t>
         </is>
       </c>
       <c r="I10" s="3" t="n">
@@ -1587,20 +1585,22 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>transit</t>
+          <t>docked</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>KRINC -&gt; VNSGN</t>
-        </is>
-      </c>
-      <c r="G19" s="2" t="n">
-        <v/>
+          <t>VNSGN (SGN03)</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>2608S</t>
+        </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>In transit, ETA 2026-09-24T15:00:00</t>
+          <t>Alongside, departs to THLCH ~2026-09-25T14:00:00</t>
         </is>
       </c>
       <c r="I19" s="3" t="n">
@@ -1965,22 +1965,20 @@
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>docked</t>
+          <t>transit</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>THBKK (BKK04)</t>
-        </is>
-      </c>
-      <c r="G25" s="2" t="inlineStr">
-        <is>
-          <t>2609N</t>
-        </is>
+          <t>THBKK -&gt; THLCH</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="n">
+        <v/>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>Alongside, departs to THLCH ~2026-09-24T14:00:00</t>
+          <t>In transit, ETA 2026-09-24T19:00:00</t>
         </is>
       </c>
       <c r="I25" s="3" t="n">
@@ -49639,7 +49637,7 @@
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
     <col width="40" customWidth="1" min="6" max="6"/>
     <col width="15" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
@@ -49668,7 +49666,7 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Old ETA (prev)</t>
+          <t>Old ETA (9-24-1300-SKED.xls)</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">

</xml_diff>

<commit_message>
Order the two port-call tiles by which happens sooner
The vessel card always rendered ETA -> THBKK before ETA -> THLCH
regardless of which one was actually next, which read as out-of-order
whenever the THLCH call came first chronologically (e.g. KMTC
GWANGYANG showing THBKK 47h away before THLCH 36h away). Added
portTilesInOrder() to compare the two ports' relevant time (the
docked-until time if currently alongside, otherwise the ETA) and put
the sooner one first.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Vessel Schedule.xlsx
+++ b/Vessel Schedule.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Full Schedule" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Early-Delay" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Full Schedule" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Early-Delay" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1255,20 +1255,22 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>nodata</t>
+          <t>docked</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="n">
-        <v/>
+          <t>VNSGN (SGN03)</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>2615N</t>
+        </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>No data in window</t>
+          <t>Alongside, departs to KRINC ~2026-09-26T13:00:00</t>
         </is>
       </c>
       <c r="I13" s="3" t="n">
@@ -1321,20 +1323,22 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>nodata</t>
+          <t>docked</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G14" s="2" t="n">
-        <v/>
+          <t>KRINC (INC08)</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>2608S</t>
+        </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>No data in window</t>
+          <t>Alongside, departs to KRPUS ~2026-09-26T12:00:00</t>
         </is>
       </c>
       <c r="I14" s="3" t="n"/>
@@ -1491,22 +1495,20 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>docked</t>
+          <t>transit</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>VNSGN (SGN03)</t>
-        </is>
-      </c>
-      <c r="G17" s="2" t="inlineStr">
-        <is>
-          <t>2609N</t>
-        </is>
+          <t>VNSGN -&gt; KRINC</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="n">
+        <v/>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>Alongside, departs to KRINC ~2026-09-25T20:00:00</t>
+          <t>In transit, ETA 2026-10-01T06:00:00</t>
         </is>
       </c>
       <c r="I17" s="3" t="n">
@@ -1949,22 +1951,20 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>docked</t>
+          <t>transit</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>VNSGN (SGN03)</t>
-        </is>
-      </c>
-      <c r="G24" s="2" t="inlineStr">
-        <is>
-          <t>2610N</t>
-        </is>
+          <t>VNSGN -&gt; KRPUS</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="n">
+        <v/>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>Alongside, departs to KRKAN ~2026-09-25T19:00:00</t>
+          <t>In transit, ETA 2026-10-01T02:00:00</t>
         </is>
       </c>
       <c r="I24" s="3" t="n">
@@ -2403,20 +2403,22 @@
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>nodata</t>
+          <t>docked</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G31" s="2" t="n">
-        <v/>
+          <t>IDJKT (JKT02)</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>2607N</t>
+        </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>No data in window</t>
+          <t>Alongside, departs to VNSGN ~2026-09-28T00:30:00</t>
         </is>
       </c>
       <c r="I31" s="3" t="n"/>
@@ -34390,7 +34392,7 @@
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
     <col width="30" customWidth="1" min="6" max="6"/>
     <col width="15" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
@@ -34419,7 +34421,7 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Old ETA (prev)</t>
+          <t>Old ETA (auto-20260925-1011-SKED.xlsx)</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">

</xml_diff>

<commit_message>
Add ETB column to the Full Schedule leg table
ETB was already in the leg data (used by the Excel export) but not
rendered in the HTML detail panel table.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Vessel Schedule.xlsx
+++ b/Vessel Schedule.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Full Schedule" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Early-Delay" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Full Schedule" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Early-Delay" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -28959,7 +28959,7 @@
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="21" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
     <col width="25" customWidth="1" min="6" max="6"/>
     <col width="15" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
@@ -28988,7 +28988,7 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Old ETA (prev)</t>
+          <t>Old ETA (9-25-1700-SKED.xls)</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">

</xml_diff>

<commit_message>
Sort currently-docked vessels by arrival time, not next future ETA
"Soonest first" was sorting a docked vessel by its next future arrival
at either port -- which for a vessel just arrived can be its *next*
rotation, weeks out -- so it ranked behind a vessel that simply hasn't
arrived yet today (e.g. SKY ORION, alongside at THBKK, sorted behind
KMTC SURABAYA arriving at THLCH in 2h). Docked vessels now sort by
dockedSince, which is always in the past, so they rank ahead of any
vessel still inbound.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Vessel Schedule.xlsx
+++ b/Vessel Schedule.xlsx
@@ -1317,22 +1317,20 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>docked</t>
+          <t>transit</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>KRINC (INC08)</t>
-        </is>
-      </c>
-      <c r="G14" s="2" t="inlineStr">
-        <is>
-          <t>2608S</t>
-        </is>
+          <t>KRINC -&gt; KRPUS</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="n">
+        <v/>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>Alongside, departs to KRPUS ~2026-09-26T12:00:00</t>
+          <t>In transit, ETA 2026-09-27T11:30:00</t>
         </is>
       </c>
       <c r="I14" s="3" t="n"/>

</xml_diff>

<commit_message>
Show Gregorian (ค.ศ.) year in Full Schedule table, not Buddhist Era
fmtDateShort was converting to a 2-digit Buddhist Era year (e.g. "69"
for พ.ศ. 2569), which read as a confusing/wrong year next to the
Gregorian dates used everywhere else on the dashboard.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Vessel Schedule.xlsx
+++ b/Vessel Schedule.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Full Schedule" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Early-Delay" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Full Schedule" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Early-Delay" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -47943,7 +47943,7 @@
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="21" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
     <col width="40" customWidth="1" min="6" max="6"/>
     <col width="15" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
@@ -47972,7 +47972,7 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Old ETA (prev)</t>
+          <t>Old ETA (auto-20260929-2041-SKED.xlsx)</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">

</xml_diff>

<commit_message>
Add a Summary view listing every vessel's current location
A third view button next to List/Calendar. Shows one compact table row
per vessel: name/code, service, status (Alongside/Sailing/No data),
current location (port+wharf, or sailing from->to), and since/ETA --
so you can see at a glance where the whole fleet is without opening
each card. Reuses earliestPortDate() for the default sort so it's
consistent with the List view: vessels alongside at THBKK/THLCH first,
then everyone else by next TH arrival. Respects the existing search
box; also sortable A-Z.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Vessel Schedule.xlsx
+++ b/Vessel Schedule.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Full Schedule" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Early-Delay" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Full Schedule" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Early-Delay" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2295,22 +2295,20 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>docked</t>
+          <t>transit</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>VNSGN (SGN03)</t>
-        </is>
-      </c>
-      <c r="G30" s="2" t="inlineStr">
-        <is>
-          <t>2607N</t>
-        </is>
+          <t>VNSGN -&gt; HKHKG</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="n">
+        <v/>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>Alongside, departs to HKHKG ~2026-10-01T07:30:00</t>
+          <t>In transit, ETA 2026-10-03T16:00:00</t>
         </is>
       </c>
       <c r="I30" s="3" t="n"/>
@@ -46825,7 +46823,7 @@
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="21" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
     <col width="40" customWidth="1" min="6" max="6"/>
     <col width="15" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
@@ -46854,7 +46852,7 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Old ETA (prev)</t>
+          <t>Old ETA (auto-20260930-1910-SKED.xlsx)</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">

</xml_diff>

<commit_message>
Use English labels throughout the Summary view
The sort dropdown and Since/ETA column had Thai text while every other
label on the page (headers, status pills) was English, inconsistent
with the rest of the Summary table.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Vessel Schedule.xlsx
+++ b/Vessel Schedule.xlsx
@@ -1357,22 +1357,20 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>docked</t>
+          <t>transit</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>KRPUS (PUS05)</t>
-        </is>
-      </c>
-      <c r="G15" s="2" t="inlineStr">
-        <is>
-          <t>2605W</t>
-        </is>
+          <t>KRPUS -&gt; KRKAN</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="n">
+        <v/>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>Alongside, departs to KRKAN ~2026-10-01T08:00:00</t>
+          <t>In transit, ETA 2026-10-01T15:00:00</t>
         </is>
       </c>
       <c r="I15" s="3" t="n"/>

</xml_diff>

<commit_message>
Hide past legs in the Summary view's Full Schedule panel
The List view's card detail panel intentionally keeps past legs
visible (greyed out, for context against delta badges), but Summary
is meant as a quick "where is it now / what's next" lookup, so past
legs there were just scroll-past clutter. renderDetailPanel() takes an
optional hidePast flag; Summary passes true, List is unchanged.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Vessel Schedule.xlsx
+++ b/Vessel Schedule.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Full Schedule" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Early-Delay" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Full Schedule" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Early-Delay" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -47885,7 +47885,7 @@
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="21" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
     <col width="40" customWidth="1" min="6" max="6"/>
     <col width="15" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
@@ -47914,7 +47914,7 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Old ETA (prev)</t>
+          <t>Old ETA (auto-20260930-2258-SKED.xlsx)</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">

</xml_diff>

<commit_message>
Show voyage number in the Summary and Calendar views
Summary gets a new Voyage column (reuses primaryVygBound(), same logic
the List view cards use). Calendar's day-detail panel gets a voyage
badge per port call, and the month-grid chip tooltip now includes it
too.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Vessel Schedule.xlsx
+++ b/Vessel Schedule.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Full Schedule" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Early-Delay" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Full Schedule" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Early-Delay" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -551,22 +551,20 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>docked</t>
+          <t>transit</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>CNSHK (SHE04)</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>2614N</t>
-        </is>
+          <t>CNSHK -&gt; TWKEL</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v/>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Alongside, departs to TWKEL ~2026-10-02T06:30:00</t>
+          <t>In transit, ETA 2026-10-03T23:00:00</t>
         </is>
       </c>
       <c r="I2" s="3" t="n">
@@ -917,24 +915,26 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>transit</t>
+          <t>docked</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>THLCH -&gt; THBKK</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="n">
-        <v/>
+          <t>THBKK (BKK01)</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>2611N</t>
+        </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>In transit, ETA 2026-10-02T06:00:00</t>
+          <t>Alongside, departs to THLCH ~2026-10-03T17:00:00</t>
         </is>
       </c>
       <c r="I8" s="3" t="n">
-        <v>46297.25</v>
+        <v>46317.79166666666</v>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
@@ -943,7 +943,7 @@
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>2611N</t>
+          <t>2612N</t>
         </is>
       </c>
       <c r="L8" s="3" t="n">
@@ -1463,22 +1463,20 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>docked</t>
+          <t>transit</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>KRINC (INC07)</t>
-        </is>
-      </c>
-      <c r="G17" s="2" t="inlineStr">
-        <is>
-          <t>2610S</t>
-        </is>
+          <t>KRINC -&gt; KRPUS</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="n">
+        <v/>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>Alongside, departs to KRPUS ~2026-10-02T07:00:00</t>
+          <t>In transit, ETA 2026-10-03T10:00:00</t>
         </is>
       </c>
       <c r="I17" s="3" t="n">
@@ -2167,20 +2165,22 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>transit</t>
+          <t>docked</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>IDJKT -&gt; IDSRG</t>
-        </is>
-      </c>
-      <c r="G28" s="2" t="n">
-        <v/>
+          <t>IDSRG (SRG02)</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>2612N</t>
+        </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>In transit, ETA 2026-10-02T08:00:00</t>
+          <t>Alongside, departs to THLCH ~2026-10-02T22:00:00</t>
         </is>
       </c>
       <c r="I28" s="3" t="n"/>
@@ -47883,7 +47883,7 @@
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="21" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
     <col width="40" customWidth="1" min="6" max="6"/>
     <col width="15" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
@@ -47912,7 +47912,7 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Old ETA (prev)</t>
+          <t>Old ETA (auto-20261001-1620-SKED.xlsx)</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">

</xml_diff>

<commit_message>
Add a route map to each vessel's Full Schedule panel
A Leaflet/OpenStreetMap map above the leg table plots every port call
in ETA order: past hops grey-dashed, upcoming hops solid teal, TH
ports highlighted, plus an estimated current position (alongside at a
port, or linearly interpolated between last departure and next ETA).
Hovering a port lists its voyage/ETA/ETD calls. Summary view's panel
hides past legs like its table does, but still links the estimated
position to the next port.

Port coordinates live in port_coords.json; the generator warns when a
schedule uses a port code missing from it. Longitudes are unwrapped
along the route so the Pacific crossing to Manzanillo (MXZLO) takes
the short way instead of spanning the whole map. Lines are straight
between ports, not real sea lanes -- the legend says so.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Vessel Schedule.xlsx
+++ b/Vessel Schedule.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Full Schedule" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Early-Delay" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Full Schedule" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Early-Delay" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1235,20 +1235,22 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>nodata</t>
+          <t>docked</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="n">
-        <v/>
+          <t>KRINC (INC07)</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>2616S</t>
+        </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>No data in window</t>
+          <t>Alongside, departs to KRPUS ~2026-10-03T15:00:00</t>
         </is>
       </c>
       <c r="I13" s="3" t="n">
@@ -2101,22 +2103,20 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>docked</t>
+          <t>transit</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>KRKAN (KAN06)</t>
-        </is>
-      </c>
-      <c r="G27" s="2" t="inlineStr">
-        <is>
-          <t>2611S</t>
-        </is>
+          <t>KRKAN -&gt; HKHKG</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="n">
+        <v/>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>Alongside, departs to HKHKG ~2026-10-02T23:00:00</t>
+          <t>In transit, ETA 2026-10-05T20:00:00</t>
         </is>
       </c>
       <c r="I27" s="3" t="n">
@@ -2167,22 +2167,20 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>docked</t>
+          <t>transit</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>IDSRG (SRG02)</t>
-        </is>
-      </c>
-      <c r="G28" s="2" t="inlineStr">
-        <is>
-          <t>2612N</t>
-        </is>
+          <t>IDSRG -&gt; THLCH</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="n">
+        <v/>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>Alongside, departs to THLCH ~2026-10-02T23:00:00</t>
+          <t>In transit, ETA 2026-10-06T16:30:00</t>
         </is>
       </c>
       <c r="I28" s="3" t="n"/>
@@ -47846,7 +47844,7 @@
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="21" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
     <col width="40" customWidth="1" min="6" max="6"/>
     <col width="15" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
@@ -47875,7 +47873,7 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Old ETA (prev)</t>
+          <t>Old ETA (auto-20261002-1532-SKED.xlsx)</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">

</xml_diff>

<commit_message>
Translate the remaining dashboard UI to English
Stats tiles, search placeholder/empty state, sort option, card
position lines, countdowns ("in ~2 days"), delay/early badges ("6h",
"1.5d"), change lines, card expand hint, port tile fallbacks, the
data-source line and calendar aria-labels were still Thai. Page lang
set to "en". The template now has no Thai text left; wharf names in
Korean come from Wharf.xls itself and are unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Vessel Schedule.xlsx
+++ b/Vessel Schedule.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Full Schedule" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Early-Delay" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Full Schedule" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Early-Delay" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2289,20 +2289,22 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>transit</t>
+          <t>docked</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>HKHKG -&gt; CNSHK</t>
-        </is>
-      </c>
-      <c r="G30" s="2" t="n">
-        <v/>
+          <t>CNSHK (SHE04)</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>2607N</t>
+        </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>In transit, ETA 2026-10-05T08:00:00</t>
+          <t>Alongside, departs to KRINC ~2026-10-07T22:00:00</t>
         </is>
       </c>
       <c r="I30" s="3" t="n"/>
@@ -47842,7 +47844,7 @@
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="21" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
     <col width="40" customWidth="1" min="6" max="6"/>
     <col width="15" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
@@ -47871,7 +47873,7 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Old ETA (prev)</t>
+          <t>Old ETA (auto-20261004-2116-SKED.xlsx)</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">

</xml_diff>

<commit_message>
Put Full Schedule above Voyage Map; add Fujairah (AEFJR) coordinates
Reordered the vessel detail panel so the leg table comes first and the
map follows it. The generator warned that MELBOURNE BRIDGE's rotation
now calls AEFJR, which wasn't in port_coords.json, so it was being
dropped from that vessel's map.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Vessel Schedule.xlsx
+++ b/Vessel Schedule.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Full Schedule" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Early-Delay" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Full Schedule" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Early-Delay" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -46579,7 +46579,7 @@
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="21" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
     <col width="40" customWidth="1" min="6" max="6"/>
     <col width="15" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
@@ -46608,7 +46608,7 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Old ETA (prev)</t>
+          <t>Old ETA (auto-20261008-2201-SKED.xlsx)</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">

</xml_diff>

<commit_message>
Berth timeline: labelled 6-hour slots, vessel name + voyage on every call
- Day header gets a second row splitting each day into 00/06/12/18
  slots; slot and day gridlines darkened (the previous 6h dashes were
  too faint to see). Scale widened to 48px per 6h (36px on phones).
- Every call now shows vessel name + voyage (plus wharf and times):
  inside the bar when it fits, measured with canvas measureText,
  otherwise as a label just right of the bar. Lanes are packed on the
  bar + label footprint so a label never runs into the next call; the
  layout re-runs once web fonts load since widths are measured. The
  vessel-code-only fallback for short Laem Chabang calls is gone.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Vessel Schedule.xlsx
+++ b/Vessel Schedule.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Full Schedule" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Early-Delay" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Full Schedule" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Early-Delay" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1413,22 +1413,20 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>docked</t>
+          <t>transit</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>KRPUS (PUS05)</t>
-        </is>
-      </c>
-      <c r="G16" s="2" t="inlineStr">
-        <is>
-          <t>2607W</t>
-        </is>
+          <t>KRPUS -&gt; CNSHA</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="n">
+        <v/>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>Alongside, departs to CNSHA ~2026-10-10T15:00:00</t>
+          <t>In transit, ETA 2026-10-12T00:00:00</t>
         </is>
       </c>
       <c r="I16" s="3" t="n"/>
@@ -46585,7 +46583,7 @@
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
     <col width="40" customWidth="1" min="6" max="6"/>
     <col width="15" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
@@ -46614,7 +46612,7 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Old ETA (prev)</t>
+          <t>Old ETA (auto-20261010-0528-SKED.xlsx)</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">

</xml_diff>

<commit_message>
Berth timeline: 4-hour slots; names always inside a solid bar
- Each day now splits into six 4-hour slots (00/04/08/12/16/20) in the
  header and gridlines; scale 40px per 4h (28px on phones).
- Short calls are still lengthened to fit vessel name + voyage, but the
  whole bar is now solid colour (the hatched tail read as "outside the
  bar"). A faint dashed tick behind the text marks the real ETD, and
  the ETB→ETD times on the bar stay exact. Dropped the unused hatch
  helper.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Vessel Schedule.xlsx
+++ b/Vessel Schedule.xlsx
@@ -2359,20 +2359,22 @@
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>transit</t>
+          <t>docked</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>KRUSN -&gt; KRINC</t>
-        </is>
-      </c>
-      <c r="G31" s="2" t="n">
-        <v/>
+          <t>KRINC (INC08)</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>2608S</t>
+        </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>In transit, ETA 2026-10-10T17:00:00</t>
+          <t>Alongside, departs to CNSHA ~2026-10-11T17:00:00</t>
         </is>
       </c>
       <c r="I31" s="3" t="n"/>

</xml_diff>

<commit_message>
Summary view: add ALL / THBKK / THLCH port filter
Picking a port lists only vessels alongside there now or with an
upcoming call there, sorts them by that port (alongside first, then by
ETA at the port; A-Z still available), and relabels the last column
"At THBKK" / "At THLCH" showing "Alongside since …" or that port's ETA
instead of the vessel's next-port ETA. Works together with the shared
search box.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Vessel Schedule.xlsx
+++ b/Vessel Schedule.xlsx
@@ -551,22 +551,20 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>docked</t>
+          <t>transit</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>KRUSN (USN01)</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>2615S</t>
-        </is>
+          <t>KRUSN -&gt; HKHKG</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v/>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Alongside, departs to HKHKG ~2026-10-10T18:00:00</t>
+          <t>In transit, ETA 2026-10-14T06:00:00</t>
         </is>
       </c>
       <c r="I2" s="3" t="n">
@@ -1465,22 +1463,20 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>docked</t>
+          <t>transit</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>VNSGN (SGN03)</t>
-        </is>
-      </c>
-      <c r="G17" s="2" t="inlineStr">
-        <is>
-          <t>2610S</t>
-        </is>
+          <t>VNSGN -&gt; THLCH</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="n">
+        <v/>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>Alongside, departs to THLCH ~2026-10-10T18:00:00</t>
+          <t>In transit, ETA 2026-10-12T11:00:00</t>
         </is>
       </c>
       <c r="I17" s="3" t="n">

</xml_diff>

<commit_message>
Add a Service filter shared by List, Calendar, Summary and Berth
One dropdown next to the search box ("All services" + each service with
its vessel count) filters every view. List/Summary match a vessel if any
of its upcoming legs is on that service, so a vessel mid service-swap
shows under both; Calendar and Berth filter per port call.

Vessel service label now comes from the leg it's on now (alongside, else
next call) instead of its oldest row, which could be a past voyage: 4
labels were stale (e.g. SAWASDEE VEGA PCI2 -> VTS). The 1-tile cap for
long-haul services also covers the new "PCI" code. View buttons wrap on
phones (Berth was cut off), and Dalian/Tianjin coordinates added for the
voyage maps.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Vessel Schedule.xlsx
+++ b/Vessel Schedule.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Full Schedule" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Early-Delay" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Full Schedule" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Early-Delay" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -729,7 +729,7 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>PVS2</t>
+          <t>KHS1</t>
         </is>
       </c>
       <c r="D5" s="2" t="n">
@@ -793,7 +793,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>ADHS</t>
+          <t>PCI2</t>
         </is>
       </c>
       <c r="D6" s="2" t="n">
@@ -853,7 +853,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>ANX</t>
+          <t>PCI</t>
         </is>
       </c>
       <c r="D7" s="2" t="n">
@@ -861,20 +861,22 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>transit</t>
+          <t>docked</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>KRPUS -&gt; KRPUS</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="n">
-        <v/>
+          <t>KRPUS (PUS05)</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>2608S</t>
+        </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>In transit, ETA 2026-10-19T13:00:00</t>
+          <t>Alongside, departs to KRKAN ~2026-10-20T13:00:00</t>
         </is>
       </c>
       <c r="I7" s="3" t="n"/>
@@ -1681,20 +1683,22 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>transit</t>
+          <t>docked</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>KRINC -&gt; CNTAO</t>
-        </is>
-      </c>
-      <c r="G20" s="2" t="n">
-        <v/>
+          <t>CNTAO (TAO04)</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>2611S</t>
+        </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>In transit, ETA 2026-10-19T14:00:00</t>
+          <t>Alongside, departs to CNSHA ~2026-10-21T03:00:00</t>
         </is>
       </c>
       <c r="I20" s="3" t="n">
@@ -2045,7 +2049,7 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>PCI2</t>
+          <t>VTS</t>
         </is>
       </c>
       <c r="D26" s="2" t="n">
@@ -45774,7 +45778,7 @@
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="21" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
     <col width="40" customWidth="1" min="6" max="6"/>
     <col width="15" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
@@ -45803,7 +45807,7 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Old ETA (prev)</t>
+          <t>Old ETA (auto-20261019-0040-SKED.xlsx)</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">

</xml_diff>

<commit_message>
Move the Service dropdown next to the Berth view button
Sits at the end of the List/Calendar/Summary/Berth button row, styled
to match those buttons, instead of beside the search box.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Vessel Schedule.xlsx
+++ b/Vessel Schedule.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Full Schedule" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Early-Delay" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Full Schedule" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Early-Delay" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1109,22 +1109,20 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>docked</t>
+          <t>transit</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>KRINC (INC08)</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="inlineStr">
-        <is>
-          <t>2608S</t>
-        </is>
+          <t>KRINC -&gt; KRPUS</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="n">
+        <v/>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>Alongside, departs to KRPUS ~2026-10-19T18:00:00</t>
+          <t>In transit, ETA 2026-10-20T19:00:00</t>
         </is>
       </c>
       <c r="I11" s="3" t="n"/>
@@ -45778,7 +45776,7 @@
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="21" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
     <col width="40" customWidth="1" min="6" max="6"/>
     <col width="15" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
@@ -45807,7 +45805,7 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Old ETA (prev)</t>
+          <t>Old ETA (auto-20261019-0501-SKED.xlsx)</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">

</xml_diff>

<commit_message>
Add light / dark theme switch
A Dark/Light button in the header toggles the whole dashboard; the
choice is saved per browser (localStorage), and a first visit follows
the device's dark-mode setting. The theme is applied by a tiny script in
<head> before first paint, so there's no flash of the wrong one.

Converted the ~40 hard-coded colours outside the palette (mostly the
berth timeline, card titles, port-tile highlight, page glow) to CSS
variables so they get dark values too; light mode renders as before.
The header band and the green/red berth bars keep their colours in both
themes; in dark the berth "now" line turns amber so it stays visible.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Vessel Schedule.xlsx
+++ b/Vessel Schedule.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Full Schedule" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Early-Delay" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Full Schedule" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Early-Delay" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -45858,7 +45858,7 @@
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="21" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
     <col width="40" customWidth="1" min="6" max="6"/>
     <col width="15" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
@@ -45887,7 +45887,7 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Old ETA (prev)</t>
+          <t>Old ETA (auto-20261025-0501-SKED.xlsx)</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">

</xml_diff>

<commit_message>
Add Changes view: ETB/ETD moves vs last update, 24h and 7 days ago
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Vessel Schedule.xlsx
+++ b/Vessel Schedule.xlsx
@@ -45858,7 +45858,7 @@
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="21" customWidth="1" min="5" max="5"/>
     <col width="40" customWidth="1" min="6" max="6"/>
     <col width="15" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
@@ -45887,7 +45887,7 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Old ETA (auto-20261025-0501-SKED.xlsx)</t>
+          <t>Old ETA (prev)</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">

</xml_diff>

<commit_message>
Short TH wharf names from wharf code.xls; List table grouped by service
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Vessel Schedule.xlsx
+++ b/Vessel Schedule.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Full Schedule" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Early-Delay" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Full Schedule" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Early-Delay" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
Weekly closing as a dashboard view (no separate page), with Copy for email
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Vessel Schedule.xlsx
+++ b/Vessel Schedule.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Full Schedule" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Early-Delay" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Full Schedule" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Early-Delay" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
Weekly closing view: themed calendar (light/dark) matching the dashboard
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Vessel Schedule.xlsx
+++ b/Vessel Schedule.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Full Schedule" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Early-Delay" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Full Schedule" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Early-Delay" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
Weekly closing: no inner scrollbar, page scroll only
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Vessel Schedule.xlsx
+++ b/Vessel Schedule.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Full Schedule" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Early-Delay" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Full Schedule" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Early-Delay" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>